<commit_message>
Add persistent activity history trail and dual-layer Vercel storage sync
</commit_message>
<xml_diff>
--- a/data/BESS_Company_Contacts_Updated1.xlsx
+++ b/data/BESS_Company_Contacts_Updated1.xlsx
@@ -2866,7 +2866,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T61"/>
+  <dimension ref="A1:U61"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -2887,7 +2887,8 @@
     <col min="17" max="17" width="30.83203125" customWidth="1"/>
     <col min="18" max="18" width="16.83203125" customWidth="1"/>
     <col min="19" max="19" width="30.83203125" customWidth="1"/>
-    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="30.83203125" customWidth="1"/>
+    <col min="21" max="21" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2949,6 +2950,9 @@
         <v>All Contacts (JSON)</v>
       </c>
       <c r="T1" t="str">
+        <v>All Activities (JSON)</v>
+      </c>
+      <c r="U1" t="str">
         <v>Last Updated</v>
       </c>
     </row>
@@ -3014,7 +3018,10 @@
         <v>[{"name":"Prashant Sharma","designation":"","mobile":"Prashant: +91 95991 86478","isPrimary":true},{"name":"Rahul Khanna","designation":"CEO","mobile":"Rahul: +91 98110 92281","isPrimary":false}]</v>
       </c>
       <c r="T2" t="str">
-        <v>2026-09-14</v>
+        <v>[{"id":"act_init_C0001","date":"2026-09-15","type":"Note / Update","text":"Dr. Rathore introduced Prashant for BESS container liquid-cooling systems and Rahul as CEO of Kabu Projects, whose LCS brand is ATMOS.\r\nHe specifically requested details for cooling a 5 MWh container.\r\nPrashant's apparent reply later described inbuilt heaters and temperature-sensor-based control.\r\nPotential outreach angle: discuss coolant qualification directly with the cooling-system team; no coolant purchase requirement was posted.","timestamp":"2026-09-15T09:18:37.847Z"}]</v>
+      </c>
+      <c r="U2" t="str">
+        <v>2026-09-15</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -3079,6 +3086,9 @@
         <v>[{"name":"Samir Patel","designation":"Chief of Technology and Operations","mobile":"Samir: +91 62923 26680","isPrimary":true},{"name":"Subhankar","designation":"BESS integrator team","mobile":"Subhankar: +91 83369 17680","isPrimary":false}]</v>
       </c>
       <c r="T3" t="str">
+        <v>[{"id":"act_init_C0002","date":"2026-09-14","type":"Note / Update","text":"Samir was introduced as the technology and operations lead, while Subhankar posted a request for cell contact system suppliers.\r\nDr. Rathore discussed a 5 GWh automated line and shared news of a 1,000 MWh NTPC order.\r\nThe chat also reports a locally developed 104.4 kWh battery pack.\r\nPotential outreach angle: request the thermal-management or procurement owner for local BESS assembly and establish who approves the coolant.","timestamp":"2026-09-15T09:15:07.365Z"}]</v>
+      </c>
+      <c r="U3" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3144,6 +3154,9 @@
         <v>[{"name":"Nirav Mehta","designation":"Vice President","mobile":"+91 98209 80208","isPrimary":true}]</v>
       </c>
       <c r="T4" t="str">
+        <v>[{"id":"act_init_C0003","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Nirav as a vice president at AmpereHour.\nA July group news digest reported the opening of a 5 GWh manufacturing and integration facility in Pune.\nThe figure is a reported manufacturing capacity, not evidence of delivered or operating projects.\nPotential outreach angle: seek an introduction to the factory procurement and thermal-design teams for coolant evaluation.","timestamp":"2026-09-15T09:15:07.365Z"}]</v>
+      </c>
+      <c r="U4" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3209,6 +3222,9 @@
         <v>[{"name":"Bharat Chhittarka","designation":"Managing Director","mobile":"+91 96654 33009","isPrimary":true}]</v>
       </c>
       <c r="T5" t="str">
+        <v>[{"id":"act_init_C0004","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Bharat as managing director and discussed a 261 kWh BESS cabinet.\r\nThe chat explicitly describes the cabinet as having a liquid-cooling system.\r\nHe also described module-level detection and fire-suppression features; these are chat descriptions, not independently checked certifications.\r\nPotential outreach angle: discuss cabinet coolant specifications, initial filling and service replacement with the design team.","timestamp":"2026-09-15T09:15:07.365Z"}]</v>
+      </c>
+      <c r="U5" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3274,6 +3290,9 @@
         <v>[{"name":"Rahul Mandal","designation":"BESS execution","mobile":"+91 87328 40104","isPrimary":true}]</v>
       </c>
       <c r="T6" t="str">
+        <v>[{"id":"act_init_C0005","date":"2026-09-14","type":"Note / Update","text":"Rahul introduced himself as looking after an 80 MW/320 MWh BESS project.\r\nDr. Rathore explicitly linked him to JSW Energy's BESS execution team.\r\nA separate June message mentions JSW at 5 GWh, but does not establish the operating status or relation to Rahul's project.\r\nPotential outreach angle: identify the project's BESS OEM, coolant approval owner and O&amp;M sourcing route.","timestamp":"2026-09-15T09:15:07.365Z"}]</v>
+      </c>
+      <c r="U6" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3339,6 +3358,9 @@
         <v>[{"name":"Shyam Shrivastava","designation":"VP Sales","mobile":"+91 96543 52855","isPrimary":true},{"name":"later described as institutional business lead","designation":"","mobile":"","isPrimary":false}]</v>
       </c>
       <c r="T7" t="str">
+        <v>[{"id":"act_init_C0006","date":"2026-09-14","type":"Note / Update","text":"Shyam reported that Invergy had recently inaugurated a BESS manufacturing facility.\r\nHe invited group members to visit and offered support for business discussions.\r\nA later group post described him as leading institutional BESS and inverter business.\r\nPotential outreach angle: ask him to connect you to thermal engineering and procurement, beginning with clarification of the stated 3GW factory capacity.","timestamp":"2026-09-15T09:15:07.365Z"}]</v>
+      </c>
+      <c r="U7" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3404,6 +3426,9 @@
         <v>[{"name":"Krishnendu Rath","designation":"BESS manufacturing / renewable energy | Introduced contacts","mobile":"+91 86553 38096","isPrimary":true},{"name":"Amit Lalani","designation":"Procurement","mobile":"7878019423","isPrimary":false},{"name":"Mithil Gandhi","designation":"HOD BESS","mobile":"9819066954","isPrimary":false}]</v>
       </c>
       <c r="T8" t="str">
+        <v>[{"id":"act_init_C0007","date":"2026-09-14","type":"Note / Update","text":"Krishnendu was introduced for renewable energy and energy storage at Waaree.\r\nA September group digest reported that Waaree had started 5.15 GWh BESS container manufacturing.\r\nThe introduction does not identify the precise Waaree legal entity responsible for coolant procurement.\r\nPotential outreach angle: request the relevant BESS factory's thermal-management and sourcing contact before discussing volumes.","timestamp":"2026-09-15T09:15:07.365Z"}]</v>
+      </c>
+      <c r="U8" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3469,6 +3494,9 @@
         <v>[{"name":"Y Bhaskara Rao","designation":"AVP","mobile":"Not stated in exported text","isPrimary":false},{"name":"Avinash Gowdnalli","designation":"Manager","mobile":"7760828480","isPrimary":true},{"name":"Sachin Barker","designation":"","mobile":"7090219767","isPrimary":false}]</v>
       </c>
       <c r="T9" t="str">
+        <v>[{"id":"act_init_C0008","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Y Bhaskara Rao as AVP of Lineage Power.\nHe later reported that a new 2,500 MWh line doubled total capacity to 5,000 MWh.\nAn August digest also describes a 100 MWh supply and commissioning-support order from Kalpa Power.\nPotential outreach angle: obtain Rao's direct contact through Dr. Rathore and ask about coolant sourcing for local battery integration.","timestamp":"2026-09-15T09:15:07.365Z"}]</v>
+      </c>
+      <c r="U9" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3534,6 +3562,9 @@
         <v>[{"name":"Pierre Andre Nutte","designation":"BESS Sales Director India/MEA","mobile":"Pierre: +33 6 07 62 83 04","isPrimary":true},{"name":"Adityan","designation":"BESS Sales &amp; Business Developer","mobile":"Adityan: +33 6 87 76 05 13","isPrimary":false}]</v>
       </c>
       <c r="T10" t="str">
+        <v>[{"id":"act_init_C0009","date":"2026-09-14","type":"Note / Update","text":"Pierre was introduced as the BESS sales director for India and MEA.\r\nAdityan's self-introduction identified SAFT as a BESS manufacturer and supplier and cited more than 10 GWh installed and contracted.\r\nThe chat does not separate the operating installed base from future contracted projects.\r\nPotential outreach angle: request the supplier-qualification team and clarify whether coolant is sourced centrally or by the local integration partner.","timestamp":"2026-09-15T09:15:07.365Z"}]</v>
+      </c>
+      <c r="U10" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3600,6 +3631,9 @@
         <v>[{"name":"Kishorsinh Zala","designation":"Chairman","mobile":"+91 99099 54615","isPrimary":false},{"name":"Dr. Hardik Patel","designation":"Chief Technology Officer (BESS R&amp;D)","mobile":"+91 98250 12345","isPrimary":false},{"name":"Amit Shah","designation":"Head of Sourcing &amp; SCM","mobile":"+91 97270 67890","isPrimary":false},{"name":"Pankaj Srivastava","designation":"COO(Chief Operating Officer)","mobile":"+91 75730 14600","isPrimary":true}]</v>
       </c>
       <c r="T11" t="str">
+        <v>[{"id":"act_init_C0010","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced the group's chairman directly.\nHis August list of Gujarat BESS assembly plants assigns Power Trac a 10 GWh capacity.\nThe post does not provide commissioning evidence, utilisation or yearly production.\nPotential outreach angle: discuss the assembly programme and seek the person responsible for liquid-cooling components and coolant sourcing.\nProduction will start from DEC'26","timestamp":"2026-09-15T09:15:07.365Z"}]</v>
+      </c>
+      <c r="U11" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3665,6 +3699,9 @@
         <v>[{"name":"Ajit Agarwal","designation":"","mobile":"Unassigned candidates: +91 97121 77777","isPrimary":true},{"name":"Tapan Agarwal","designation":"","mobile":"+91 70271 39999","isPrimary":false},{"name":"Prakash","designation":"","mobile":"+91 90995 11572","isPrimary":false}]</v>
       </c>
       <c r="T12" t="str">
+        <v>[{"id":"act_init_C0011","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced three Castrochem contacts together and located the company in Palanpur.\r\nA later assembly-plant list gives Castrochem a 2 GWh capacity.\r\nThree phone numbers appear around the introduction, but the export does not map each number to a named person.\r\nPotential outreach angle: first confirm the identities, factory location and commissioning status, then ask about coolant qualification.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U12" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3730,6 +3767,9 @@
         <v>[{"name":"Jitendra Kumar","designation":"also tagged Jitender Kumar","mobile":"+91 99102 19897","isPrimary":true}]</v>
       </c>
       <c r="T13" t="str">
+        <v>[{"id":"act_init_C0012","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Jitendra as a Hithium contact and directed another member to him.\r\nA later message mentions a 6.25 MWh AC block and 1,175 Ah cells in a Saudi Arabia context.\r\nThose figures describe a product discussion rather than this contact's company-wide manufacturing or installed capacity.\r\nPotential outreach angle: establish the Indian supplier-approval route and which team controls cooling-fluid specifications.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U13" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3795,6 +3835,9 @@
         <v>[{"name":"Rajiv Saini","designation":"described by Dr. Rathore as REPT India business-development contact","mobile":"Not stated in exported text","isPrimary":true}]</v>
       </c>
       <c r="T14" t="str">
+        <v>[{"id":"act_init_C0013","date":"2026-09-14","type":"Note / Update","text":"Rajiv was introduced in association with REPT and discussed Bitek products in the group.\r\nThe chat includes 5 MWh container discussions and his claim that Bitek with REPT had completed more than 1 GWh.\r\nThe export records Rajiv's removal from the group on 11 September; direct contact will need to come from your saved contacts or an introduction.\r\nPotential outreach angle: verify his current company role and thermal-system sourcing responsibility before proceeding.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U14" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3860,6 +3903,9 @@
         <v>[{"name":"Prahlad Mittal","designation":"","mobile":"Prahlad: +91 98878 80968","isPrimary":true},{"name":"Rakesh Kumar","designation":"","mobile":"Rakesh: not recovered","isPrimary":false}]</v>
       </c>
       <c r="T15" t="str">
+        <v>[{"id":"act_init_C0014","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Prahlad and Rakesh in connection with Oriana Power/True RE.\r\nPrahlad later signed a technical discussion as being from Oriana Power Limited, Noida.\r\nHis contribution addressed BESS sizing, operating conditions, efficiency and losses, indicating a technical project contact.\r\nPotential outreach angle: ask who specifies the project's BESS cooling system and whether coolant procurement rests with Oriana or its OEM.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U15" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3925,6 +3971,9 @@
         <v>[{"name":"Anoop Mehra","designation":"O&amp;M Head","mobile":"+91 94609 38390","isPrimary":true}]</v>
       </c>
       <c r="T16" t="str">
+        <v>[{"id":"act_init_C0015","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Anoop as ACME's O&amp;M head and a matching contact card is in the ZIP.\r\nA later group digest reports a 300 MW/1,200 MWh award and an approximately 15 GWh PPA-signed storage pipeline.\r\nThese figures should not be treated as current operating capacity or Anoop's personal project scope.\r\nPotential outreach angle: discuss approved coolant maintenance, replacement and warranty procedures with the O&amp;M team.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U16" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -3990,6 +4039,9 @@
         <v>[{"name":"Andrew Curry","designation":"VP Manufacturing and Engineering","mobile":"Andrew: +91 89767 83588","isPrimary":true},{"name":"Dr. Björn Mårlid","designation":"CEO","mobile":"CEO: not recovered","isPrimary":false}]</v>
       </c>
       <c r="T17" t="str">
+        <v>[{"id":"act_init_C0016","date":"2026-09-14","type":"Note / Update","text":"Andrew was introduced as VP Manufacturing and Engineering.\r\nOther posts identify Dr. Björn Mårlid as CEO and refer to the company's sodium-ion battery team.\r\nThe chat discusses their participation in BESS, PCS and EMS training but gives no firm production capacity.\r\nPotential outreach angle: ask the manufacturing team whether their system design uses a compatible liquid coolant and who owns qualification.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U17" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4055,6 +4107,9 @@
         <v>[{"name":"Dino","designation":"Energy-storage supplier contact | Introduced contacts","mobile":"+86 159 5040 1225","isPrimary":true}]</v>
       </c>
       <c r="T18" t="str">
+        <v>[{"id":"act_init_C0017","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Dino as a WHES representative.\r\nHe tagged the same number in a discussion of energy-management algorithms and full-stack technology.\r\nThe available introduction contains no factory capacity, installed base or business address.\r\nPotential outreach angle: establish the company's container/cabinet offering and route to the thermal-management or purchasing team.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U18" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4120,6 +4175,9 @@
         <v>[{"name":"Tushar Gupta","designation":"BESS / EV charging | Introduced contacts","mobile":"+91 95820 73337","isPrimary":true}]</v>
       </c>
       <c r="T19" t="str">
+        <v>[{"id":"act_init_C0018","date":"2026-09-14","type":"Note / Update","text":"Tushar's signed post describes Servotech's EV charger business and a BESS-plus-charger supply to NHAI.\r\nHe also mentions larger prototypes being developed for coal-mining companies.\r\nThe chat provides no numerical capacity for those battery systems.\r\nPotential outreach angle: discuss prototype thermal-management requirements and ask for the engineer or buyer handling coolant selection.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U19" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4185,6 +4243,9 @@
         <v>[{"name":"Prathamesh","designation":"Design Engineer","mobile":"+91 95451 14696","isPrimary":true}]</v>
       </c>
       <c r="T20" t="str">
+        <v>[{"id":"act_init_C0019","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Prathamesh as a design engineer at Neuron Energy.\r\nThe introduction is useful as a technical entry point rather than proof of a live purchase requirement.\r\nNo project size, installed capacity or factory address accompanies the introduction.\r\nPotential outreach angle: ask about liquid-cooled battery designs and the specification/testing process for a new coolant supplier.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U20" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4250,6 +4311,9 @@
         <v>[{"name":"Saurabh Srivastava","designation":"BESS manufacturing / integration | Introduced contacts","mobile":"+91 98922 24218","isPrimary":true}]</v>
       </c>
       <c r="T21" t="str">
+        <v>[{"id":"act_init_C0020","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore welcomed Saurabh and asked him to brief the group about LNT BESS.\r\nIn the same message he requested a visit to the Chennai plant.\r\nThis establishes a plant-related introduction but does not establish the plant's capacity or Saurabh's designation.\r\nPotential outreach angle: request the BESS manufacturing, thermal-design or supplier-development contact at the Chennai facility.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U21" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4315,6 +4379,9 @@
         <v>[{"name":"Mohd Imran","designation":"BESS business contact | Introduced contacts","mobile":"+91 95997 58634","isPrimary":true}]</v>
       </c>
       <c r="T22" t="str">
+        <v>[{"id":"act_init_C0021","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore explicitly introduced Mohd Imran for Samsung C&amp;T BESS.\r\nThe number is supported by the same-time add event and a subsequent greeting.\r\nNo project capacity or office address is supplied in the introduction.\r\nPotential outreach angle: establish whether his team specifies BESS equipment, procures complete systems or can refer you to its cooling-system supplier.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U22" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4380,6 +4447,9 @@
         <v>[{"name":"Dr. Ravi","designation":"Founder Director","mobile":"+91 90330 00000","isPrimary":true}]</v>
       </c>
       <c r="T23" t="str">
+        <v>[{"id":"act_init_C0022","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Dr. Ravi as Rocket Power's founder director.\r\nHe also described delivering BESS training to the Rocket Power team in Rajkot.\r\nThe chat does not give a manufacturing line size or installed battery portfolio for the firm.\r\nPotential outreach angle: establish the company's BESS assembly plans and whether its products require externally sourced coolant.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U23" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4445,6 +4515,9 @@
         <v>[{"name":"Li Xueyi","designation":"Custom LFP ESS/BESS supplier | Introduced contacts","mobile":"+86 132 8326 1678","isPrimary":true}]</v>
       </c>
       <c r="T24" t="str">
+        <v>[{"id":"act_init_C0023","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Li Xueyi with a description of customised LFP batteries for ESS/BESS projects.\r\nThe introduction states that the company provides technical support and pre-sales, sales and after-sales service.\r\nNo product energy range, factory capacity or address is included.\r\nPotential outreach angle: identify which configurations use liquid cooling and whether the firm sources coolant or buys prefilled systems.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U24" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4510,6 +4583,9 @@
         <v>[{"name":"LIU XiaoXiao","designation":"Nora","mobile":"+86 181 5019 6050","isPrimary":true}]</v>
       </c>
       <c r="T25" t="str">
+        <v>[{"id":"act_init_C0024","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore welcomed CATL and tagged Nora as the relevant group contact.\r\nA separate member's SNEC post describes a 20-foot, 3 MWh sodium-ion container.\r\nThat example is not a capacity figure for Nora's business unit or an Indian factory.\r\nPotential outreach angle: request the formal coolant supplier-qualification route and ask whether India-related procurement is local or centralised.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U25" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4575,6 +4651,9 @@
         <v>[{"name":"Dheeraj","designation":"Energy / BESS prospect | Introduced contacts","mobile":"+91 89895 16992","isPrimary":true}]</v>
       </c>
       <c r="T26" t="str">
+        <v>[{"id":"act_init_C0025","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Dheeraj as a contact from LNJ Bhilwara Energy.\r\nThe introduction gives no designation, BESS project capacity or business address.\r\nHistorical thermal-power references elsewhere in the group are not treated as this firm's BESS capacity.\r\nPotential outreach angle: establish his current storage-project responsibilities and obtain the relevant OEM or procurement contact.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U26" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4640,6 +4719,9 @@
         <v>[{"name":"Sushil Bansal","designation":"Founder and Managing Director","mobile":"+91 98601 44666","isPrimary":true}]</v>
       </c>
       <c r="T27" t="str">
+        <v>[{"id":"act_init_C0026","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Sushil as founder and managing director.\r\nSeveral messages describe BESS training planned or delivered for the Novasys team in Nagpur.\r\nTraining activity is evidence of interest in storage, not evidence of an installed BESS manufacturing line.\r\nPotential outreach angle: ask about the company's BESS rollout and obtain the responsible technical/procurement lead.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U27" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4705,6 +4787,9 @@
         <v>[{"name":"Tanveer Chawla","designation":"Director","mobile":"Tanveer: +91 95740 77777","isPrimary":true},{"name":"Kirit Shah and Ankul Kanala","designation":"Directors","mobile":"others: not reliably mapped","isPrimary":false}]</v>
       </c>
       <c r="T28" t="str">
+        <v>[{"id":"act_init_C0027","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Tanveer and subsequently welcomed directors Kirit Shah and Ankul Kanala.\r\nHis itinerary describes a multi-day BESS training engagement with Krushnam Infra in Ahmedabad.\r\nThe chat does not quantify its factory capacity or installed storage projects.\r\nPotential outreach angle: ask about forthcoming BESS projects and who selects the cooling-system package.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U28" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4770,6 +4855,9 @@
         <v>[{"name":"Jitendra Singh Shekhawat","designation":"Managing Director","mobile":"+91 98750 00011","isPrimary":true}]</v>
       </c>
       <c r="T29" t="str">
+        <v>[{"id":"act_init_C0028","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Jitendra as managing director of Adhiraj Group.\r\nHe also described advising the group on a BESS project in a Rajasthan expo discussion.\r\nNo reliable energy capacity for that project is provided in the selected source messages.\r\nPotential outreach angle: determine the project's execution stage and whether coolant is specified by the developer or the contracted BESS integrator.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U29" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4835,6 +4923,9 @@
         <v>[{"name":"Vishal Dhruve","designation":"Managing Director","mobile":"+91 97264 40058","isPrimary":true}]</v>
       </c>
       <c r="T30" t="str">
+        <v>[{"id":"act_init_C0029","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Vishal as managing director of Total Solar Technology in Ahmedabad.\r\nThe introduction gives a senior business entry point but no BESS deployment or manufacturing figure.\r\nIts direct coolant demand therefore remains unqualified.\r\nPotential outreach angle: ask whether the firm is moving into liquid-cooled BESS assembly or can introduce its battery-system supplier.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U30" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4900,6 +4991,9 @@
         <v>[{"name":"Karthikeyan Subramanian","designation":"Director","mobile":"+91 73959 53335","isPrimary":true}]</v>
       </c>
       <c r="T31" t="str">
+        <v>[{"id":"act_init_C0030","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Karthikeyan as a director of ACE RenewTech.\r\nThe available welcome post does not describe a specific battery factory or project.\r\nIt also provides no business address or quantified storage capacity.\r\nPotential outreach angle: first qualify the firm's BESS role and request a connection to the relevant system integrator or procurement team.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U31" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -4965,6 +5059,9 @@
         <v>[{"name":"Nishi Chandra","designation":"Solar / BESS sales prospect | Introduced contacts","mobile":"+91 96504 43724","isPrimary":true}]</v>
       </c>
       <c r="T32" t="str">
+        <v>[{"id":"act_init_C0031","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Nishi as a Loom Solar contact near the end of the export.\r\nThe contact thanked him, but the subsequent product images are omitted from the text export.\r\nConsequently, product sizes and coolant compatibility cannot be recovered from those images.\r\nPotential outreach angle: ask about liquid-cooled commercial storage offerings and the relevant OEM sourcing contact.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U32" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5030,6 +5127,9 @@
         <v>[{"name":"Priyansh Mohan","designation":"Founder CEO","mobile":"Not stated in exported text","isPrimary":true}]</v>
       </c>
       <c r="T33" t="str">
+        <v>[{"id":"act_init_C0032","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Priyansh as founder and CEO of an iron-battery storage start-up.\r\nThe post describes a different storage technology from conventional lithium-ion BESS.\r\nNo production capacity, project size or cooling-fluid requirement is established in the text.\r\nPotential outreach angle: obtain a direct introduction and qualify the cooling architecture before presenting your coolant.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U33" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5095,6 +5195,9 @@
         <v>[{"name":"Jitendra Singh Ranawat","designation":"Vice President RE+BESS","mobile":"Not stated in exported text","isPrimary":true}]</v>
       </c>
       <c r="T34" t="str">
+        <v>[{"id":"act_init_C0033","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Jitendra as GIPCL's vice president for RE and BESS.\r\nThe title makes him a possible project-level introduction route.\r\nA different earlier post tags an unnamed GIPCL vice president, but it does not prove that number belongs to Jitendra.\r\nPotential outreach angle: ask Dr. Rathore for a direct introduction and identify the contracted BESS and cooling-system OEMs.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U34" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5160,6 +5263,9 @@
         <v>[{"name":"Hari Om Vishwakarma","designation":"Flow-battery project contact | Introduced contacts","mobile":"+91 82750 45064","isPrimary":true}]</v>
       </c>
       <c r="T35" t="str">
+        <v>[{"id":"act_init_C0034","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore welcomed Hari Om in connection with a 100 MWh vanadium redox flow battery.\r\nThe technology and project size are explicitly stated, but the project stage and site are not.\r\nThis should not be treated as a confirmed lithium-ion coolant application.\r\nPotential outreach angle: ask whether the project has an external thermal-management loop relevant to your product and who supplies it.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U35" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5225,6 +5331,9 @@
         <v>[{"name":"Sardar Bahadori","designation":"BESS builder | Introduced contacts","mobile":"+36 30 116 0355","isPrimary":true}]</v>
       </c>
       <c r="T36" t="str">
+        <v>[{"id":"act_init_C0035","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Sardar as a BESS builder from Hungary.\r\nA matching number appears in the add event and ensuing greeting.\r\nThe legal company name, factory size, installed base and full address are absent.\r\nPotential outreach angle: first obtain the company profile and establish whether it builds liquid-cooled systems suitable for your coolant.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U36" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5290,6 +5399,9 @@
         <v>[{"name":"Nitin Sharma","designation":"","mobile":"Nitin: +91 97699 80963","isPrimary":true},{"name":"Nitesh Bhutada","designation":"","mobile":"Nitesh: not recovered","isPrimary":false}]</v>
       </c>
       <c r="T37" t="str">
+        <v>[{"id":"act_init_C0036","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore described visiting Newen's works and observing PCS assembly and testing.\r\nHe introduced the management team and separately referred a member to Nitesh Bhutada for PCS and DC-to-DC converters.\r\nThe ZIP contains Nitin Sharma's named contact card.\r\nPotential outreach angle: use this as a technical referral route to BESS integrators; direct coolant buying is not established.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U37" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5355,6 +5467,9 @@
         <v>[{"name":"Chetan Gunjal","designation":"BESS assembly-line equipment | Additional leads / referral routes","mobile":"Not stated in exported text","isPrimary":true}]</v>
       </c>
       <c r="T38" t="str">
+        <v>[{"id":"act_init_C0037","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Chetan as a contact for BESS assembly lines.\r\nAn earlier message associates Maestrotech with SPML's 5 GWh automated line.\r\nThat figure describes a customer's line, not Maestrotech's own battery factory output.\r\nPotential outreach angle: discuss introductions to new BESS assembly customers and whether coolant filling/testing is part of the equipment scope.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U38" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5420,6 +5535,9 @@
         <v>[{"name":"Nikhil Aroda","designation":"BESS assembly equipment | Additional leads / referral routes","mobile":"+91 98187 42050","isPrimary":true}]</v>
       </c>
       <c r="T39" t="str">
+        <v>[{"id":"act_init_C0038","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Nikhil for BESS assembly-plant setup.\r\nAnother post mentions a laser-welding machine from Shinop Encore.\r\nThe introduction provides no manufacturing capacity or installed battery portfolio.\r\nPotential outreach angle: seek referrals to new battery-assembly facilities and ask where coolant filling fits in their process.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U39" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5485,6 +5603,9 @@
         <v>[{"name":"Gaurav Kochar","designation":"PCS supplier | Additional leads / referral routes","mobile":"+91 98028 80441","isPrimary":true}]</v>
       </c>
       <c r="T40" t="str">
+        <v>[{"id":"act_init_C0039","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Gaurav as a Fimer PCS contact.\r\nNo specific BESS project or factory size appears in the introduction.\r\nA PCS relationship does not itself establish that the contact buys battery coolant.\r\nPotential outreach angle: ask for relevant BESS integrator or thermal-equipment contacts if direct product compatibility is not present.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U40" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5550,6 +5671,9 @@
         <v>[{"name":"Rakesh Kumar","designation":"Technical and Services","mobile":"+91 84212 45837","isPrimary":true}]</v>
       </c>
       <c r="T41" t="str">
+        <v>[{"id":"act_init_C0040","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced Rakesh as a technical and services contact at Deye.\r\nThe welcome message does not identify a specific liquid-cooled BESS product or project.\r\nNo factory capacity or business address is supplied.\r\nPotential outreach angle: establish whether his service portfolio includes coolant-bearing systems and request the responsible procurement team.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U41" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5615,6 +5739,9 @@
         <v>[{"name":"India Head","designation":"name not stated","mobile":"+91 89688 18307","isPrimary":true}]</v>
       </c>
       <c r="T42" t="str">
+        <v>[{"id":"act_init_C0041","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore introduced the Lux Power India head without naming the person.\r\nThe nearby group-add event supplies a candidate contact number.\r\nThe introduction provides no numerical storage capacity or cooling-system details.\r\nPotential outreach angle: qualify the product portfolio and request an introduction to a relevant BESS integration partner.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U42" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5680,6 +5807,9 @@
         <v>[{"name":"Not stated in exported text","designation":"BESS assembly prospect | Additional leads / referral routes","mobile":"Not stated in exported text","isPrimary":true}]</v>
       </c>
       <c r="T43" t="str">
+        <v>[{"id":"act_init_C0042","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore included Ddev Plastiks in his list of Gujarat BESS assembly plants.\r\nHe assigned it 5 GWh and separately referred to a relationship with the company.\r\nThe text does not establish actual output or a named procurement contact.\r\nPotential outreach angle: ask Dr. Rathore to introduce the BESS manufacturing or thermal-management head.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U43" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5745,6 +5875,9 @@
         <v>[{"name":"Not stated in exported text","designation":"Planned BESS OEM | Additional leads / referral routes","mobile":"Not stated in exported text","isPrimary":true}]</v>
       </c>
       <c r="T44" t="str">
+        <v>[{"id":"act_init_C0043","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore listed Samarth at 2 GWh in August.\r\nHis later September message states that Shree Samarth had ordered a line and would soon become a BESS OEM.\r\nThe later wording is treated as a planned/ordered line rather than an operating factory.\r\nPotential outreach angle: seek an introduction while coolant specifications and initial suppliers may still be under selection.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U44" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5810,6 +5943,9 @@
         <v>[{"name":"Not stated in exported text","designation":"BESS assembly prospect | Additional leads / referral routes","mobile":"Not stated in exported text","isPrimary":true}]</v>
       </c>
       <c r="T45" t="str">
+        <v>[{"id":"act_init_C0044","date":"2026-09-14","type":"Note / Update","text":"Earth Span appears in Dr. Rathore's list of BESS assembly plants.\r\nThe stated capacity is 2 GWh, with no additional project or factory evidence in the relevant text.\r\nNo individual contact or mobile number is reliably attached to this firm.\r\nPotential outreach angle: request the exact company name and factory contact through Dr. Rathore before qualifying coolant demand.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U45" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5875,6 +6011,9 @@
         <v>[{"name":"Not stated in exported text","designation":"BESS assembly prospect | Additional leads / referral routes","mobile":"Not stated in exported text","isPrimary":true}]</v>
       </c>
       <c r="T46" t="str">
+        <v>[{"id":"act_init_C0045","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore's assembly-plant list includes Grace Power at 3 GWh.\r\nThe message does not name a representative or identify the legal entity.\r\nA separate Grace Renewable Energy contact appears in the chat, but the text does not establish that the two names refer to the same company.\r\nPotential outreach angle: ask Dr. Rathore to resolve the entity and introduce its battery manufacturing team.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U46" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -5940,6 +6079,9 @@
         <v>[{"name":"Not stated in exported text","designation":"Planned BESS OEM | Additional leads / referral routes","mobile":"Not stated in exported text","isPrimary":true}]</v>
       </c>
       <c r="T47" t="str">
+        <v>[{"id":"act_init_C0046","date":"2026-09-14","type":"Note / Update","text":"Dr. Rathore said Sky Energy had ordered a BESS line and would soon become an OEM.\r\nThe same post refers to it as one of his clients.\r\nNeither the line capacity nor a named company contact is provided.\r\nPotential outreach angle: request an introduction for early coolant specification discussions, subject to confirming the firm's identity and project stage.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U47" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6005,6 +6147,9 @@
         <v>[{"name":"Harsh Bagadia","designation":"Battery procurement lead | Additional leads / referral routes","mobile":"+91 75739 27000","isPrimary":true}]</v>
       </c>
       <c r="T48" t="str">
+        <v>[{"id":"act_init_C0047","date":"2026-09-14","type":"Note / Update","text":"Harsh posted a named request to procure 6,400 units of 100 Ah cells.\r\nThis is direct evidence of battery procurement activity, although the application and cooling design are not specified.\r\nThe cell quantity is not converted into MWh because the post does not give the required voltage/configuration.\r\nPotential outreach angle: qualify whether the cells are for liquid-cooled BESS and identify the coolant decision maker.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U48" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6070,6 +6215,9 @@
         <v>[{"name":"Praveen","designation":"BESS project / procurement referral | Additional leads / referral routes","mobile":"+91 90000 13241","isPrimary":true}]</v>
       </c>
       <c r="T49" t="str">
+        <v>[{"id":"act_init_C0048","date":"2026-09-14","type":"Note / Update","text":"The export includes a contact card labelled Praveen Bondada.\r\nA later group news digest refers to Bondada Renewable BESS supply agreements with the Pace Digitek group.\r\nThe card does not state Praveen's designation or establish that he controls those projects.\r\nPotential outreach angle: confirm his role and request the BESS procurement or O&amp;M contact.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U49" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6132,6 +6280,9 @@
         <v>[{"name":"Venkat Rajaraman","designation":"MD","mobile":"8978990444","isPrimary":true},{"name":"Kethan Yadagiri","designation":"","mobile":"8309389300","isPrimary":false}]</v>
       </c>
       <c r="T50" t="str">
+        <v>[{"id":"act_init_C0049","date":"2026-09-14","type":"Note / Update","text":"Highest-priority contact: liquid-cooled modules are already in production; coolant/dielectric fluid is a live BoM item now.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U50" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6194,6 +6345,9 @@
         <v/>
       </c>
       <c r="T51" t="str">
+        <v>[{"id":"act_init_C0050","date":"2026-09-14","type":"Note / Update","text":"Approach as a live product-spec discussion — ask which coolant/fluid is currently used in the containerised line and whether they source it or buy pre-filled units.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U51" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6256,6 +6410,9 @@
         <v/>
       </c>
       <c r="T52" t="str">
+        <v>[{"id":"act_init_C0051","date":"2026-09-14","type":"Note / Update","text":"Established manufacturer with in-house R&amp;D — worth qualifying whether their BESS/ESS line is air- or liquid-cooled before pitching.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U52" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6318,6 +6475,9 @@
         <v/>
       </c>
       <c r="T53" t="str">
+        <v>[{"id":"act_init_C0052","date":"2026-09-14","type":"Note / Update","text":"Mahashakti (utility-scale) is the coolant-relevant SKU — confirm its container-level thermal design before outreach.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U53" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6380,6 +6540,9 @@
         <v/>
       </c>
       <c r="T54" t="str">
+        <v>[{"id":"act_init_C0053","date":"2026-09-14","type":"Note / Update","text":"Existing pack-assembly operation is a live coolant-spec conversation now; the larger integration facility is a 2026-27 design-in window (tracked separately).","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U54" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6442,6 +6605,9 @@
         <v/>
       </c>
       <c r="T55" t="str">
+        <v>[{"id":"act_init_C0054","date":"2026-09-14","type":"Note / Update","text":"Long-lead but very high-volume account — approach via the BESS/cell manufacturing division once commissioning completes, expected H2 2026.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U55" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6504,6 +6670,9 @@
         <v/>
       </c>
       <c r="T56" t="str">
+        <v>[{"id":"act_init_C0055","date":"2026-09-14","type":"Note / Update","text":"Early-stage design-in opportunity — engage before Phase 1 BoM is finalized (FY26-27 window).","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U56" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6566,6 +6735,9 @@
         <v/>
       </c>
       <c r="T57" t="str">
+        <v>[{"id":"act_init_C0056","date":"2026-09-14","type":"Note / Update","text":"Solar-major diversifying into BESS manufacturing — track FY27 commissioning for coolant-spec conversations.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U57" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6628,6 +6800,9 @@
         <v/>
       </c>
       <c r="T58" t="str">
+        <v>[{"id":"act_init_C0057","date":"2026-09-14","type":"Note / Update","text":"Very early stage (term sheet only, Sep 2026) — good for relationship-building ahead of formal BoM decisions.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U58" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6690,6 +6865,9 @@
         <v/>
       </c>
       <c r="T59" t="str">
+        <v>[{"id":"act_init_C0058","date":"2026-09-14","type":"Note / Update","text":"Track for commissioning-date updates; too early for firm BoM discussion.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U59" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6752,6 +6930,9 @@
         <v/>
       </c>
       <c r="T60" t="str">
+        <v>[{"id":"act_init_C0059","date":"2026-09-14","type":"Note / Update","text":"Adani buys/deploys containers rather than manufacturing them — the coolant decision sits with its chosen BESS/container OEM (not yet identified) rather than with Adani directly. Worth establishing which OEM(s) are supplying the containers.","timestamp":"2026-09-15T09:15:07.366Z"}]</v>
+      </c>
+      <c r="U60" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
@@ -6814,12 +6995,15 @@
         <v>[{"name":"Shekhar Bhosle","designation":"Senior CFD EngineerBESS manufacturer | Introduced contacts","mobile":"7709333859","isPrimary":false},{"name":"Amit Alurkar","designation":"Head","mobile":"9822094950","isPrimary":true},{"name":"Sujay Khare","designation":"Manager","mobile":"9559083502","isPrimary":false}]</v>
       </c>
       <c r="T61" t="str">
+        <v/>
+      </c>
+      <c r="U61" t="str">
         <v>2026-09-14</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>